<commit_message>
Agenda Excel: add Sponsors Summary tab; fix parser to capture meal-row sponsors (Atlantic Emergency Solutions, MSA-Globe)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BCOC_2026_Agenda.xlsx
+++ b/BCOC_2026_Agenda.xlsx
@@ -7,11 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCOC 2026 Agenda" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agenda" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sponsors Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BCOC 2026 Agenda'!$A$1:$J$70</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'BCOC 2026 Agenda'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agenda'!$A$1:$J$70</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Agenda'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sponsors Summary'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +43,12 @@
       <b val="1"/>
       <color rgb="0014213D"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +90,21 @@
         <fgColor rgb="00FDEDEA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006B7280"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8962E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -111,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -162,6 +183,27 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -622,7 +664,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Check-In &amp; Registration</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
@@ -654,7 +700,11 @@
           <t>Exhibit</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Vendor / Sponsor Exhibit Hall Setup</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
@@ -770,7 +820,11 @@
           <t>Exhibit</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Vendor / Sponsor Exhibit Hall Setup (continued)</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
@@ -1134,7 +1188,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Group Photo — All Attendees</t>
+        </is>
+      </c>
       <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr"/>
@@ -1172,7 +1230,11 @@
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Atlantic Emergency Solutions *Platinum</t>
+        </is>
+      </c>
       <c r="I16" s="3" t="inlineStr"/>
       <c r="J16" s="3" t="inlineStr"/>
     </row>
@@ -1323,7 +1385,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Session</t>
+          <t>Social</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1366,7 +1428,11 @@
           <t>Exhibit</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr"/>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Vendor / Sponsor Exhibit Hall Open</t>
+        </is>
+      </c>
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
@@ -1602,7 +1668,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr"/>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Break — Visit Vendor &amp; Sponsor Exhibit Hall</t>
+        </is>
+      </c>
       <c r="G27" s="6" t="inlineStr"/>
       <c r="H27" s="6" t="inlineStr"/>
       <c r="I27" s="6" t="inlineStr"/>
@@ -1728,7 +1798,11 @@
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr"/>
-      <c r="H30" s="6" t="inlineStr"/>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Atlantic Emergency Solutions *Platinum / MSA-Globe *Gold</t>
+        </is>
+      </c>
       <c r="I30" s="6" t="inlineStr"/>
       <c r="J30" s="6" t="inlineStr"/>
     </row>
@@ -1802,7 +1876,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr"/>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Book Signing: Dr. I. David Daniels — "Psychosocial Hazards Are Real!" / Visit Vendor Exhibit Hall</t>
+        </is>
+      </c>
       <c r="G32" s="6" t="inlineStr"/>
       <c r="H32" s="6" t="inlineStr"/>
       <c r="I32" s="6" t="inlineStr"/>
@@ -1970,7 +2048,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Daily Wrap-up — Visit Vendor Exhibit Hall</t>
+        </is>
+      </c>
       <c r="G36" s="6" t="inlineStr"/>
       <c r="H36" s="6" t="inlineStr"/>
       <c r="I36" s="6" t="inlineStr"/>
@@ -2046,7 +2128,11 @@
           <t>Exhibit</t>
         </is>
       </c>
-      <c r="F38" s="9" t="inlineStr"/>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>Vendor / Sponsor Exhibit Hall Open</t>
+        </is>
+      </c>
       <c r="G38" s="9" t="inlineStr"/>
       <c r="H38" s="9" t="inlineStr"/>
       <c r="I38" s="9" t="inlineStr"/>
@@ -2078,7 +2164,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr"/>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>Networking Breakfast</t>
+        </is>
+      </c>
       <c r="G39" s="9" t="inlineStr"/>
       <c r="H39" s="9" t="inlineStr"/>
       <c r="I39" s="9" t="inlineStr"/>
@@ -2154,7 +2244,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F41" s="9" t="inlineStr"/>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>Coffee Break — Visit Vendor Exhibit Hall</t>
+        </is>
+      </c>
       <c r="G41" s="9" t="inlineStr"/>
       <c r="H41" s="9" t="inlineStr"/>
       <c r="I41" s="9" t="inlineStr"/>
@@ -2274,7 +2368,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F44" s="9" t="inlineStr"/>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>Networking Break — Visit Vendor Exhibit Hall</t>
+        </is>
+      </c>
       <c r="G44" s="9" t="inlineStr"/>
       <c r="H44" s="9" t="inlineStr"/>
       <c r="I44" s="9" t="inlineStr"/>
@@ -2312,7 +2410,11 @@
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr"/>
-      <c r="H45" s="9" t="inlineStr"/>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>Atlantic Emergency Solutions *Platinum</t>
+        </is>
+      </c>
       <c r="I45" s="9" t="inlineStr"/>
       <c r="J45" s="9" t="inlineStr"/>
     </row>
@@ -2422,7 +2524,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F48" s="9" t="inlineStr"/>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>Refresh Break — Visit Vendor Exhibit Hall</t>
+        </is>
+      </c>
       <c r="G48" s="9" t="inlineStr"/>
       <c r="H48" s="9" t="inlineStr"/>
       <c r="I48" s="9" t="inlineStr"/>
@@ -2542,7 +2648,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr"/>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Networking Break — Visit Vendor Exhibit Hall</t>
+        </is>
+      </c>
       <c r="G51" s="9" t="inlineStr"/>
       <c r="H51" s="9" t="inlineStr"/>
       <c r="I51" s="9" t="inlineStr"/>
@@ -2614,7 +2724,11 @@
           <t>Exhibit</t>
         </is>
       </c>
-      <c r="F53" s="12" t="inlineStr"/>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>Vendor / Sponsor Exhibit Hall Open</t>
+        </is>
+      </c>
       <c r="G53" s="12" t="inlineStr"/>
       <c r="H53" s="12" t="inlineStr"/>
       <c r="I53" s="12" t="inlineStr"/>
@@ -2774,7 +2888,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F57" s="12" t="inlineStr"/>
+      <c r="F57" s="12" t="inlineStr">
+        <is>
+          <t>Coffee &amp; Networking Break</t>
+        </is>
+      </c>
       <c r="G57" s="12" t="inlineStr"/>
       <c r="H57" s="12" t="inlineStr"/>
       <c r="I57" s="12" t="inlineStr"/>
@@ -2892,7 +3010,11 @@
         </is>
       </c>
       <c r="G60" s="12" t="inlineStr"/>
-      <c r="H60" s="12" t="inlineStr"/>
+      <c r="H60" s="14" t="inlineStr">
+        <is>
+          <t>Atlantic Emergency Solutions *Platinum</t>
+        </is>
+      </c>
       <c r="I60" s="12" t="inlineStr"/>
       <c r="J60" s="12" t="inlineStr"/>
     </row>
@@ -3178,7 +3300,11 @@
           <t>Break</t>
         </is>
       </c>
-      <c r="F67" s="15" t="inlineStr"/>
+      <c r="F67" s="15" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="G67" s="15" t="inlineStr"/>
       <c r="H67" s="15" t="inlineStr"/>
       <c r="I67" s="15" t="inlineStr"/>
@@ -3312,4 +3438,238 @@
   <autoFilter ref="A1:J70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t># Items</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sponsored Items (Date · Time — Session)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>FirstNet</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>Elite Premier</t>
+        </is>
+      </c>
+      <c r="C2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>• Mon, Aug 3 · 9:30 - 11:00 AM — "From Trauma to Triumph, But Still I Lead"
+• Tue, Aug 4 · 8:30 - 9:30 AM — Leading Through What You Don't Know: Executive Blind Spots in Times of Challenge
+• Tue, Aug 4 · 9:30 - 9:35 AM — FirstNet Sponsor Presentation
+• Tue, Aug 4 · 7:00 - 10:00 PM — Opening Reception Hospitality Night
+• Thu, Aug 6 · 7:00 - 10:00 PM — Comedy Showcase + Karaoke Night</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Atlantic Emergency Solutions</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>Platinum</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>• Mon, Aug 3 · 12:00 - 1:00 PM — Lunch Break
+• Tue, Aug 4 · 12:15 - 1:15 PM — Luncheon
+• Wed, Aug 5 · 12:00 - 1:00 PM — Lunch
+• Thu, Aug 6 · 12:00 - 1:30 PM — Sponsor Appreciation Luncheon</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Pierce</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>Platinum</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>• Fri, Aug 7 · 6:30 - 8:00 PM — Oratorical Contest — $10,000 Scholarship</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>REV Fire Group</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>Platinum</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>• Mon, Aug 3 · 7:00 - 8:15 AM — Registration &amp; Networking Breakfast
+• Tue, Aug 4 · 8:00 - 8:30 AM — Harmony Breakfast
+• Wed, Aug 5 · 8:30 - 9:30 AM — Global Perspectives on Executive Fire Service Leadership
+• Thu, Aug 6 · 1:30 - 2:30 PM — The Seven Pillars of Modern Leadership: Integrating Public Safety Competencies as Black Chief Officers</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>1-800-BoardUp</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>• Mon, Aug 3 · 7:00 - 8:15 AM — Registration &amp; Networking Breakfast</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>American Wood Council</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>• Mon, Aug 3 · 7:00 - 10:00 PM — Welcome Reception</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>MSA-Globe</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>• Tue, Aug 4 · 12:15 - 1:15 PM — Luncheon</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Sutphen</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>• Tue, Aug 4 · 8:00 - 8:30 AM — Harmony Breakfast
+• Wed, Aug 5 · 5:00 - 7:00 PM — Evening Activities / Evening Buffet</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>CPSE</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>• Tue, Aug 4 · 3:15 - 3:45 PM — CPSE Credentialing</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Oratorical: replace Capt. Chatman with Chief John Reed; normalize 'Pierce' to 'Pierce Manufacturing' across agenda + sponsor page; regenerate Excel
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BCOC_2026_Agenda.xlsx
+++ b/BCOC_2026_Agenda.xlsx
@@ -3387,12 +3387,12 @@
       </c>
       <c r="G69" s="15" t="inlineStr">
         <is>
-          <t>Capt. Chatman (AFD)</t>
+          <t>Chief John Reed</t>
         </is>
       </c>
       <c r="H69" s="17" t="inlineStr">
         <is>
-          <t>Pierce *Platinum</t>
+          <t>Pierce Manufacturing *Platinum</t>
         </is>
       </c>
       <c r="I69" s="15" t="inlineStr"/>
@@ -3527,7 +3527,7 @@
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
         <is>
-          <t>Pierce</t>
+          <t>Pierce Manufacturing</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Set closing keynote speaker to Chief Michael J. Monds (Syracuse FD) across all areas: flipbook (row, cards, closing footer), binder, session details, bios (headshot + full bio), Excel
Replaces the TBD 'Special Presentation (Closing Keynote)' Friday 9:30-11:00 AM slot with Chief Monds' session 'Straight From a Fire Lieutenant to the Fire Chief'

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BCOC_2026_Agenda.xlsx
+++ b/BCOC_2026_Agenda.xlsx
@@ -1670,7 +1670,7 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Break — Visit Vendor &amp; Sponsor Exhibit Hall</t>
+          <t>Book Signing: Chief John Alston — "Leading Fearlessly" / Visit Vendor &amp; Sponsor Exhibit Hall</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr"/>
@@ -3217,21 +3217,25 @@
       </c>
       <c r="E65" s="16" t="inlineStr">
         <is>
-          <t>Keynote</t>
+          <t>Closing Keynote</t>
         </is>
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
-          <t>Special Presentation (Closing Keynote)</t>
+          <t>Straight From a Fire Lieutenant to the Fire Chief: Leadership Lessons, Breaking Barriers, and Preparing for the Chief's Office</t>
         </is>
       </c>
       <c r="G65" s="15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Chief Michael J. Monds, Syracuse Fire Department (NY)</t>
         </is>
       </c>
       <c r="H65" s="15" t="inlineStr"/>
-      <c r="I65" s="15" t="inlineStr"/>
+      <c r="I65" s="15" t="inlineStr">
+        <is>
+          <t>Syracuse Fire Chief Michael J. Monds shares his journey from Lieutenant to becoming the first Black Fire Chief in his department's 150-year history — practical guidance on preparing for the chief's office, leading with authenticity, and building credibility, resilience, and integrity.</t>
+        </is>
+      </c>
       <c r="J65" s="15" t="inlineStr"/>
     </row>
     <row r="66">

</xml_diff>